<commit_message>
add AEB cycle availability extraction and run_setting enum wiring
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73D50A2-EB51-E446-BE50-2DBAA8CF77B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0468B100-1968-AE41-81E3-82FB0C0CFB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="1160" windowWidth="34200" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
     <sheet name="calParam" sheetId="9" r:id="rId2"/>
     <sheet name="graphSpec" sheetId="3" r:id="rId3"/>
     <sheet name="KPI" sheetId="6" r:id="rId4"/>
-    <sheet name="overallKPI" sheetId="8" r:id="rId5"/>
+    <sheet name="cycleKPI" sheetId="8" r:id="rId5"/>
     <sheet name="markerShapes" sheetId="5" r:id="rId6"/>
     <sheet name="lineColors" sheetId="4" r:id="rId7"/>
   </sheets>
@@ -997,7 +997,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1033,7 +1033,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -2161,19 +2160,19 @@
       <c r="X7" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="Y7" s="19">
+      <c r="Y7" s="18">
         <v>60</v>
       </c>
-      <c r="Z7" s="19">
+      <c r="Z7" s="18">
         <v>65</v>
       </c>
-      <c r="AA7" s="19">
+      <c r="AA7" s="18">
         <v>70</v>
       </c>
-      <c r="AB7" s="19">
+      <c r="AB7" s="18">
         <v>70</v>
       </c>
-      <c r="AC7" s="19">
+      <c r="AC7" s="18">
         <v>70</v>
       </c>
     </row>
@@ -2725,25 +2724,25 @@
       <c r="X26" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="Y26" s="18">
+      <c r="Y26" s="17">
         <v>85</v>
       </c>
-      <c r="Z26" s="18">
+      <c r="Z26" s="17">
         <v>85</v>
       </c>
-      <c r="AA26" s="18">
+      <c r="AA26" s="17">
         <v>85</v>
       </c>
-      <c r="AB26" s="18">
+      <c r="AB26" s="17">
         <v>85</v>
       </c>
-      <c r="AC26" s="18">
+      <c r="AC26" s="17">
         <v>85</v>
       </c>
-      <c r="AD26" s="18">
+      <c r="AD26" s="17">
         <v>85</v>
       </c>
-      <c r="AE26" s="18">
+      <c r="AE26" s="17">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add FCW cycle availability extraction and fix cycleKPI export merging
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0468B100-1968-AE41-81E3-82FB0C0CFB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E375F086-DA8F-694A-A508-ED180FAA3125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17520" yWindow="700" windowWidth="16680" windowHeight="20460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="293">
   <si>
     <t>Reference</t>
   </si>
@@ -912,6 +912,18 @@
   </si>
   <si>
     <t>Throttle</t>
+  </si>
+  <si>
+    <t>runSetting</t>
+  </si>
+  <si>
+    <t>inputHealthy</t>
+  </si>
+  <si>
+    <t>precondBlk</t>
+  </si>
+  <si>
+    <t>abort</t>
   </si>
 </sst>
 </file>
@@ -4619,7 +4631,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5705F2F5-A4FE-CE49-A935-9D51D28B5CFA}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -4668,7 +4680,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -4685,12 +4697,12 @@
         <v>269</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>289</v>
       </c>
       <c r="C5" t="s">
         <v>70</v>
@@ -4698,16 +4710,13 @@
       <c r="D5" t="s">
         <v>77</v>
       </c>
-      <c r="E5" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>266</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>267</v>
+        <v>290</v>
       </c>
       <c r="C6" t="s">
         <v>70</v>
@@ -4715,16 +4724,13 @@
       <c r="D6" t="s">
         <v>77</v>
       </c>
-      <c r="E6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>274</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="C7" t="s">
         <v>70</v>
@@ -4732,16 +4738,13 @@
       <c r="D7" t="s">
         <v>77</v>
       </c>
-      <c r="E7" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>275</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>267</v>
+        <v>292</v>
       </c>
       <c r="C8" t="s">
         <v>70</v>
@@ -4749,8 +4752,205 @@
       <c r="D8" t="s">
         <v>77</v>
       </c>
-      <c r="E8" t="s">
+    </row>
+    <row r="9" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B9" t="s">
+        <v>267</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B10" t="s">
+        <v>289</v>
+      </c>
+      <c r="C10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B11" t="s">
+        <v>290</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" t="s">
+        <v>291</v>
+      </c>
+      <c r="C12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" t="s">
+        <v>292</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>266</v>
+      </c>
+      <c r="B14" t="s">
+        <v>267</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>266</v>
+      </c>
+      <c r="B15" t="s">
+        <v>289</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>266</v>
+      </c>
+      <c r="B16" t="s">
+        <v>290</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>266</v>
+      </c>
+      <c r="B17" t="s">
+        <v>291</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>266</v>
+      </c>
+      <c r="B18" t="s">
+        <v>292</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>274</v>
+      </c>
+      <c r="B19" t="s">
+        <v>267</v>
+      </c>
+      <c r="C19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>275</v>
+      </c>
+      <c r="B20" t="s">
+        <v>267</v>
+      </c>
+      <c r="C20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" t="s">
         <v>273</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add unit-converted signals for cycle KPIs and refactor AEB availability logic to use precondBlk only
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E375F086-DA8F-694A-A508-ED180FAA3125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928F1B05-1BB0-824C-A48D-A04D3159A5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17520" yWindow="700" windowWidth="16680" windowHeight="20460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8760" yWindow="700" windowWidth="24240" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="296">
   <si>
     <t>Reference</t>
   </si>
@@ -857,12 +857,6 @@
     <t>aeb availability</t>
   </si>
   <si>
-    <t>fcw availability</t>
-  </si>
-  <si>
-    <t>eba availability</t>
-  </si>
-  <si>
     <t>lsaeb warning availability</t>
   </si>
   <si>
@@ -924,6 +918,21 @@
   </si>
   <si>
     <t>abort</t>
+  </si>
+  <si>
+    <t>PedalPosProSuppression</t>
+  </si>
+  <si>
+    <t>SteeringWheelAngle</t>
+  </si>
+  <si>
+    <t>SteeringWheelAngleRate</t>
+  </si>
+  <si>
+    <t>YawRate</t>
+  </si>
+  <si>
+    <t>LatAccel</t>
   </si>
 </sst>
 </file>
@@ -1848,13 +1857,13 @@
   <sheetData>
     <row r="2" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="J2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="X2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.2">
@@ -1865,12 +1874,12 @@
         <v>9</v>
       </c>
       <c r="X3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -1891,7 +1900,7 @@
         <v>100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
@@ -1930,7 +1939,7 @@
         <v>250</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Y4" s="1">
         <v>0</v>
@@ -1950,7 +1959,7 @@
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C5" s="1">
         <v>42</v>
@@ -1971,7 +1980,7 @@
         <v>11</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="K5" s="1">
         <v>360</v>
@@ -2010,7 +2019,7 @@
         <v>60</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="Y5" s="17">
         <v>50</v>
@@ -2030,7 +2039,7 @@
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
@@ -2051,7 +2060,7 @@
         <v>80</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -2090,7 +2099,7 @@
         <v>80</v>
       </c>
       <c r="X6" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Y6" s="14">
         <v>0</v>
@@ -2110,7 +2119,7 @@
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C7" s="1">
         <v>12</v>
@@ -2131,7 +2140,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="K7" s="1">
         <v>220</v>
@@ -2170,7 +2179,7 @@
         <v>55</v>
       </c>
       <c r="X7" s="14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="Y7" s="18">
         <v>60</v>
@@ -2190,7 +2199,7 @@
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C8" s="14">
         <v>5</v>
@@ -2211,7 +2220,7 @@
         <v>80</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K8" s="14">
         <v>5</v>
@@ -2257,7 +2266,7 @@
     </row>
     <row r="9" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C9" s="14">
         <v>40</v>
@@ -2278,7 +2287,7 @@
         <v>18</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="K9" s="14">
         <v>430</v>
@@ -2340,7 +2349,7 @@
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
@@ -2361,7 +2370,7 @@
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C15" s="1">
         <v>5</v>
@@ -2382,7 +2391,7 @@
         <v>100</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K15" s="1">
         <v>5</v>
@@ -2409,7 +2418,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="X15" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Y15" s="1">
         <v>0</v>
@@ -2429,7 +2438,7 @@
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C16" s="1">
         <v>4</v>
@@ -2450,7 +2459,7 @@
         <v>4</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="K16" s="1">
         <v>100</v>
@@ -2477,7 +2486,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="X16" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="Y16" s="1">
         <v>20</v>
@@ -2497,7 +2506,7 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C17" s="1">
         <v>5</v>
@@ -2518,7 +2527,7 @@
         <v>80</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
@@ -2557,7 +2566,7 @@
         <v>80</v>
       </c>
       <c r="X17" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Y17" s="14">
         <v>0</v>
@@ -2577,7 +2586,7 @@
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C18" s="1">
         <v>1.7</v>
@@ -2598,7 +2607,7 @@
         <v>5.2</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="K18" s="14">
         <v>580</v>
@@ -2637,7 +2646,7 @@
         <v>240</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="Y18" s="14">
         <v>55</v>
@@ -2657,7 +2666,7 @@
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B19" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C19" s="14">
         <v>5</v>
@@ -2680,7 +2689,7 @@
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B20" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C20" s="14">
         <v>2.8</v>
@@ -2703,12 +2712,12 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X24" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X25" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="Y25" s="1">
         <v>0</v>
@@ -2734,7 +2743,7 @@
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X26" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="Y26" s="17">
         <v>85</v>
@@ -4631,7 +4640,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5705F2F5-A4FE-CE49-A935-9D51D28B5CFA}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -4680,7 +4689,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -4697,12 +4706,12 @@
         <v>269</v>
       </c>
     </row>
-    <row r="5" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C5" t="s">
         <v>70</v>
@@ -4711,12 +4720,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C6" t="s">
         <v>70</v>
@@ -4725,12 +4734,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C7" t="s">
         <v>70</v>
@@ -4739,12 +4748,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C8" t="s">
         <v>70</v>
@@ -4753,12 +4762,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
       <c r="C9" t="s">
         <v>70</v>
@@ -4766,16 +4775,13 @@
       <c r="D9" t="s">
         <v>77</v>
       </c>
-      <c r="E9" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>177</v>
+        <v>266</v>
       </c>
       <c r="B10" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="C10" t="s">
         <v>70</v>
@@ -4784,12 +4790,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>266</v>
       </c>
       <c r="B11" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C11" t="s">
         <v>70</v>
@@ -4798,12 +4804,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>266</v>
       </c>
       <c r="B12" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C12" t="s">
         <v>70</v>
@@ -4812,12 +4818,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>266</v>
       </c>
       <c r="B13" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -4826,12 +4832,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>266</v>
       </c>
       <c r="B14" t="s">
-        <v>267</v>
+        <v>290</v>
       </c>
       <c r="C14" t="s">
         <v>70</v>
@@ -4839,16 +4845,13 @@
       <c r="D14" t="s">
         <v>77</v>
       </c>
-      <c r="E14" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B15" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="C15" t="s">
         <v>70</v>
@@ -4856,13 +4859,16 @@
       <c r="D15" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E15" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B16" t="s">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="C16" t="s">
         <v>70</v>
@@ -4870,87 +4876,28 @@
       <c r="D16" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>266</v>
-      </c>
+      <c r="E16" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>291</v>
-      </c>
-      <c r="C17" t="s">
-        <v>70</v>
-      </c>
-      <c r="D17" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>266</v>
-      </c>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>292</v>
-      </c>
-      <c r="C18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D18" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>274</v>
-      </c>
+        <v>288</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>267</v>
-      </c>
-      <c r="C19" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>275</v>
-      </c>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>267</v>
-      </c>
-      <c r="C20" t="s">
-        <v>70</v>
-      </c>
-      <c r="D20" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B21" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
         <v>290</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B23" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B24" t="s">
-        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
unify MDF signal access via get_signal across event and KPI calculators
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928F1B05-1BB0-824C-A48D-A04D3159A5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B545C4-79BE-1C4D-ABF3-E64E09451E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8760" yWindow="700" windowWidth="24240" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36540" yWindow="4880" windowWidth="24240" windowHeight="14460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="297">
   <si>
     <t>Reference</t>
   </si>
@@ -933,6 +933,9 @@
   </si>
   <si>
     <t>LatAccel</t>
+  </si>
+  <si>
+    <t>LowSpeed</t>
   </si>
 </sst>
 </file>
@@ -2746,7 +2749,7 @@
         <v>280</v>
       </c>
       <c r="Y26" s="17">
-        <v>85</v>
+        <v>2</v>
       </c>
       <c r="Z26" s="17">
         <v>85</v>
@@ -4778,10 +4781,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>266</v>
+        <v>91</v>
       </c>
       <c r="B10" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="C10" t="s">
         <v>70</v>

</xml_diff>

<commit_message>
Rename AEB availability KPI keys to ROVAvail/VALAvail
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D9DD88-1510-E846-B459-536CCE22407D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AAF9285-0F80-B149-86DB-9D0EF37466F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37360" yWindow="2220" windowWidth="31940" windowHeight="19140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="290">
   <si>
     <t>Reference</t>
   </si>
@@ -845,9 +845,6 @@
     <t>feature</t>
   </si>
   <si>
-    <t>EBA</t>
-  </si>
-  <si>
     <t>AvailDistPct</t>
   </si>
   <si>
@@ -857,18 +854,6 @@
     <t>aeb availability</t>
   </si>
   <si>
-    <t>lsaeb warning availability</t>
-  </si>
-  <si>
-    <t>lsaeb actuation availability</t>
-  </si>
-  <si>
-    <t>CPM_WRN</t>
-  </si>
-  <si>
-    <t>CPM_ACT</t>
-  </si>
-  <si>
     <t>Yaw_rate</t>
   </si>
   <si>
@@ -908,12 +893,6 @@
     <t>Throttle</t>
   </si>
   <si>
-    <t>precondBlk</t>
-  </si>
-  <si>
-    <t>abort</t>
-  </si>
-  <si>
     <t>PedalPosProSuppression</t>
   </si>
   <si>
@@ -932,10 +911,10 @@
     <t>LowSpeed</t>
   </si>
   <si>
-    <t>aebROVAvail</t>
-  </si>
-  <si>
-    <t>aebVALAvail</t>
+    <t>ROVAvail</t>
+  </si>
+  <si>
+    <t>VALAvail</t>
   </si>
 </sst>
 </file>
@@ -1860,13 +1839,13 @@
   <sheetData>
     <row r="2" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="J2" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="X2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.2">
@@ -1877,12 +1856,12 @@
         <v>9</v>
       </c>
       <c r="X3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -1903,7 +1882,7 @@
         <v>100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
@@ -1942,7 +1921,7 @@
         <v>250</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="Y4" s="1">
         <v>0</v>
@@ -1962,7 +1941,7 @@
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C5" s="1">
         <v>42</v>
@@ -1983,7 +1962,7 @@
         <v>11</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="K5" s="1">
         <v>360</v>
@@ -2022,7 +2001,7 @@
         <v>60</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="Y5" s="17">
         <v>50</v>
@@ -2042,7 +2021,7 @@
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
@@ -2063,7 +2042,7 @@
         <v>80</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -2102,7 +2081,7 @@
         <v>80</v>
       </c>
       <c r="X6" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="Y6" s="14">
         <v>0</v>
@@ -2122,7 +2101,7 @@
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C7" s="1">
         <v>12</v>
@@ -2143,7 +2122,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="K7" s="1">
         <v>220</v>
@@ -2182,7 +2161,7 @@
         <v>55</v>
       </c>
       <c r="X7" s="14" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="Y7" s="18">
         <v>60</v>
@@ -2202,7 +2181,7 @@
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C8" s="14">
         <v>5</v>
@@ -2223,7 +2202,7 @@
         <v>80</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="K8" s="14">
         <v>5</v>
@@ -2269,7 +2248,7 @@
     </row>
     <row r="9" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C9" s="14">
         <v>40</v>
@@ -2290,7 +2269,7 @@
         <v>18</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="K9" s="14">
         <v>430</v>
@@ -2352,7 +2331,7 @@
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
@@ -2373,7 +2352,7 @@
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C15" s="1">
         <v>5</v>
@@ -2394,7 +2373,7 @@
         <v>100</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="K15" s="1">
         <v>5</v>
@@ -2421,7 +2400,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="X15" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="Y15" s="1">
         <v>0</v>
@@ -2441,7 +2420,7 @@
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C16" s="1">
         <v>4</v>
@@ -2462,7 +2441,7 @@
         <v>4</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="K16" s="1">
         <v>100</v>
@@ -2489,7 +2468,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="X16" s="1" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="Y16" s="1">
         <v>20</v>
@@ -2509,7 +2488,7 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C17" s="1">
         <v>5</v>
@@ -2530,7 +2509,7 @@
         <v>80</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
@@ -2569,7 +2548,7 @@
         <v>80</v>
       </c>
       <c r="X17" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="Y17" s="14">
         <v>0</v>
@@ -2589,7 +2568,7 @@
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C18" s="1">
         <v>1.7</v>
@@ -2610,7 +2589,7 @@
         <v>5.2</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="K18" s="14">
         <v>580</v>
@@ -2649,7 +2628,7 @@
         <v>240</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="Y18" s="14">
         <v>55</v>
@@ -2669,7 +2648,7 @@
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B19" s="14" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C19" s="14">
         <v>5</v>
@@ -2692,7 +2671,7 @@
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B20" s="14" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C20" s="14">
         <v>2.8</v>
@@ -2715,12 +2694,12 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X24" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X25" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="Y25" s="1">
         <v>0</v>
@@ -2746,7 +2725,7 @@
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X26" s="1" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="Y26" s="17">
         <v>2</v>
@@ -4643,7 +4622,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5705F2F5-A4FE-CE49-A935-9D51D28B5CFA}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -4678,7 +4657,7 @@
         <v>188</v>
       </c>
       <c r="E2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -4697,7 +4676,7 @@
         <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C4" t="s">
         <v>70</v>
@@ -4706,7 +4685,7 @@
         <v>77</v>
       </c>
       <c r="E4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -4714,7 +4693,7 @@
         <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="C5" t="s">
         <v>70</v>
@@ -4728,7 +4707,7 @@
         <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="C6" t="s">
         <v>70</v>
@@ -4742,7 +4721,7 @@
         <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="C7" t="s">
         <v>70</v>
@@ -4756,7 +4735,7 @@
         <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="C8" t="s">
         <v>70</v>
@@ -4770,7 +4749,7 @@
         <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C9" t="s">
         <v>70</v>
@@ -4784,7 +4763,7 @@
         <v>91</v>
       </c>
       <c r="B10" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="C10" t="s">
         <v>70</v>
@@ -4798,7 +4777,7 @@
         <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="C11" t="s">
         <v>70</v>
@@ -4812,7 +4791,7 @@
         <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="C12" t="s">
         <v>70</v>
@@ -4823,10 +4802,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" t="s">
         <v>266</v>
-      </c>
-      <c r="B13" t="s">
-        <v>287</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -4834,13 +4813,16 @@
       <c r="D13" t="s">
         <v>77</v>
       </c>
+      <c r="E13" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>266</v>
+        <v>177</v>
       </c>
       <c r="B14" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C14" t="s">
         <v>70</v>
@@ -4851,10 +4833,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>272</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>267</v>
+        <v>283</v>
       </c>
       <c r="C15" t="s">
         <v>70</v>
@@ -4862,16 +4844,13 @@
       <c r="D15" t="s">
         <v>77</v>
       </c>
-      <c r="E15" t="s">
-        <v>270</v>
-      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>273</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>267</v>
+        <v>284</v>
       </c>
       <c r="C16" t="s">
         <v>70</v>
@@ -4879,8 +4858,75 @@
       <c r="D16" t="s">
         <v>77</v>
       </c>
-      <c r="E16" t="s">
-        <v>271</v>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B17" t="s">
+        <v>285</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B18" t="s">
+        <v>286</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" t="s">
+        <v>287</v>
+      </c>
+      <c r="C19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>177</v>
+      </c>
+      <c r="B20" t="s">
+        <v>288</v>
+      </c>
+      <c r="C20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>177</v>
+      </c>
+      <c r="B21" t="s">
+        <v>289</v>
+      </c>
+      <c r="C21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify config/signal handling and streamline MF4 extraction
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B81D1F5-D925-0440-9253-DA804E4949F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8C32DF-EC28-A647-856B-5C2CB3E99585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37360" yWindow="2220" windowWidth="31940" windowHeight="19140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37360" yWindow="2220" windowWidth="31940" windowHeight="19140" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="10" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="405">
   <si>
     <t>Reference</t>
   </si>
@@ -611,12 +611,6 @@
   </si>
   <si>
     <t>name of the mdf chunk</t>
-  </si>
-  <si>
-    <t>AebKpiExtractor</t>
-  </si>
-  <si>
-    <t>FcwKpiExtractor</t>
   </si>
   <si>
     <t>WINDOW_S</t>
@@ -1258,6 +1252,15 @@
   </si>
   <si>
     <t>aebDegradation</t>
+  </si>
+  <si>
+    <t>AebEventKpiExtractor</t>
+  </si>
+  <si>
+    <t>FcwEventKpiExtractor</t>
+  </si>
+  <si>
+    <t>fcw availability</t>
   </si>
 </sst>
 </file>
@@ -1712,13 +1715,13 @@
   <sheetData>
     <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>290</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>292</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>146</v>
@@ -1729,13 +1732,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" t="s">
         <v>293</v>
-      </c>
-      <c r="B2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C2" t="s">
-        <v>295</v>
       </c>
       <c r="D2" t="s">
         <v>147</v>
@@ -1743,13 +1746,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B3" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C3" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D3" t="s">
         <v>147</v>
@@ -1757,47 +1760,47 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>296</v>
+      </c>
+      <c r="B4" t="s">
+        <v>297</v>
+      </c>
+      <c r="C4" t="s">
         <v>298</v>
-      </c>
-      <c r="B4" t="s">
-        <v>299</v>
-      </c>
-      <c r="C4" t="s">
-        <v>300</v>
       </c>
       <c r="D4" t="s">
         <v>147</v>
       </c>
       <c r="E4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C5" t="s">
         <v>302</v>
-      </c>
-      <c r="B5" t="s">
-        <v>303</v>
-      </c>
-      <c r="C5" t="s">
-        <v>304</v>
       </c>
       <c r="D5" t="s">
         <v>147</v>
       </c>
       <c r="E5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D6" t="s">
         <v>147</v>
@@ -1805,13 +1808,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>306</v>
+      </c>
+      <c r="B7" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7" t="s">
         <v>308</v>
-      </c>
-      <c r="B7" t="s">
-        <v>309</v>
-      </c>
-      <c r="C7" t="s">
-        <v>310</v>
       </c>
       <c r="D7" t="s">
         <v>147</v>
@@ -1819,13 +1822,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C8" t="s">
         <v>311</v>
-      </c>
-      <c r="B8" t="s">
-        <v>312</v>
-      </c>
-      <c r="C8" t="s">
-        <v>313</v>
       </c>
       <c r="D8" t="s">
         <v>147</v>
@@ -1833,64 +1836,64 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B9" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C9" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D9" t="s">
         <v>147</v>
       </c>
       <c r="E9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B10" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D10" t="s">
         <v>147</v>
       </c>
       <c r="E10" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B11" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C11" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D11" t="s">
         <v>147</v>
       </c>
       <c r="E11" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>320</v>
+      </c>
+      <c r="B12" t="s">
+        <v>321</v>
+      </c>
+      <c r="C12" t="s">
         <v>322</v>
-      </c>
-      <c r="B12" t="s">
-        <v>323</v>
-      </c>
-      <c r="C12" t="s">
-        <v>324</v>
       </c>
       <c r="D12" t="s">
         <v>147</v>
@@ -1898,13 +1901,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B13" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C13" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D13" t="s">
         <v>157</v>
@@ -1912,13 +1915,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B14" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D14" t="s">
         <v>157</v>
@@ -1926,13 +1929,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B15" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C15" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D15" t="s">
         <v>147</v>
@@ -1940,111 +1943,111 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C16" t="s">
+        <v>330</v>
+      </c>
+      <c r="D16" t="s">
         <v>331</v>
-      </c>
-      <c r="C16" t="s">
-        <v>332</v>
-      </c>
-      <c r="D16" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B17" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C17" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D17" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B18" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C18" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D18" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B19" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C19" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D19" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>338</v>
+      </c>
+      <c r="B20" t="s">
+        <v>339</v>
+      </c>
+      <c r="C20" t="s">
         <v>340</v>
       </c>
-      <c r="B20" t="s">
-        <v>341</v>
-      </c>
-      <c r="C20" t="s">
-        <v>342</v>
-      </c>
       <c r="D20" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B21" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C21" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B22" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C22" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D22" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>344</v>
+      </c>
+      <c r="B23" t="s">
+        <v>345</v>
+      </c>
+      <c r="C23" t="s">
         <v>346</v>
-      </c>
-      <c r="B23" t="s">
-        <v>347</v>
-      </c>
-      <c r="C23" t="s">
-        <v>348</v>
       </c>
       <c r="D23" t="s">
         <v>147</v>
@@ -2052,13 +2055,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B24" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C24" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D24" t="s">
         <v>147</v>
@@ -2066,13 +2069,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B25" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C25" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D25" t="s">
         <v>147</v>
@@ -2080,27 +2083,27 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B26" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C26" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D26" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>353</v>
+      </c>
+      <c r="B27" t="s">
+        <v>354</v>
+      </c>
+      <c r="C27" t="s">
         <v>355</v>
-      </c>
-      <c r="B27" t="s">
-        <v>356</v>
-      </c>
-      <c r="C27" t="s">
-        <v>357</v>
       </c>
       <c r="D27" t="s">
         <v>147</v>
@@ -2108,13 +2111,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B28" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C28" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D28" t="s">
         <v>147</v>
@@ -2122,13 +2125,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B29" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C29" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D29" t="s">
         <v>157</v>
@@ -2136,13 +2139,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B30" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C30" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D30" t="s">
         <v>157</v>
@@ -2150,13 +2153,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B31" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C31" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D31" t="s">
         <v>157</v>
@@ -2164,13 +2167,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B32" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C32" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D32" t="s">
         <v>157</v>
@@ -2178,13 +2181,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B33" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C33" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D33" t="s">
         <v>157</v>
@@ -2192,13 +2195,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B34" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C34" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D34" t="s">
         <v>157</v>
@@ -2206,13 +2209,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B35" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C35" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D35" t="s">
         <v>157</v>
@@ -2220,13 +2223,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B36" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C36" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D36" t="s">
         <v>157</v>
@@ -2234,13 +2237,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B37" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C37" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D37" t="s">
         <v>157</v>
@@ -2248,13 +2251,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B38" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C38" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D38" t="s">
         <v>147</v>
@@ -2262,13 +2265,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>376</v>
+      </c>
+      <c r="B39" t="s">
         <v>378</v>
       </c>
-      <c r="B39" t="s">
-        <v>380</v>
-      </c>
       <c r="C39" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D39" t="s">
         <v>147</v>
@@ -2276,13 +2279,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B40" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C40" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D40" t="s">
         <v>157</v>
@@ -2290,13 +2293,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B41" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C41" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D41" t="s">
         <v>157</v>
@@ -2304,69 +2307,69 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B42" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C42" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D42" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B43" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C43" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D43" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B44" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C44" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D44" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B45" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C45" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D45" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>391</v>
+      </c>
+      <c r="B46" t="s">
+        <v>392</v>
+      </c>
+      <c r="C46" t="s">
         <v>393</v>
-      </c>
-      <c r="B46" t="s">
-        <v>394</v>
-      </c>
-      <c r="C46" t="s">
-        <v>395</v>
       </c>
       <c r="D46" t="s">
         <v>147</v>
@@ -2374,13 +2377,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B47" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C47" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D47" t="s">
         <v>147</v>
@@ -2388,13 +2391,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B48" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C48" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D48" t="s">
         <v>147</v>
@@ -2402,13 +2405,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B49" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C49" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D49" t="s">
         <v>157</v>
@@ -2416,16 +2419,16 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B50" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C50" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D50" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -2495,7 +2498,7 @@
         <v>157</v>
       </c>
       <c r="E3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F3" t="s">
         <v>174</v>
@@ -2503,7 +2506,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -2518,12 +2521,12 @@
         <v>158</v>
       </c>
       <c r="F4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B5">
         <v>3</v>
@@ -2538,7 +2541,7 @@
         <v>159</v>
       </c>
       <c r="F5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -2552,10 +2555,10 @@
         <v>157</v>
       </c>
       <c r="E6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="F6" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2575,7 +2578,7 @@
         <v>153</v>
       </c>
       <c r="F7" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2595,12 +2598,12 @@
         <v>154</v>
       </c>
       <c r="F8" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B9">
         <v>0.32</v>
@@ -2612,10 +2615,10 @@
         <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F9" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2635,7 +2638,7 @@
         <v>155</v>
       </c>
       <c r="F10" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -2655,12 +2658,12 @@
         <v>156</v>
       </c>
       <c r="F11" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B12">
         <v>-25</v>
@@ -2672,15 +2675,15 @@
         <v>183</v>
       </c>
       <c r="E12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F12" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B13">
         <v>-20</v>
@@ -2692,15 +2695,15 @@
         <v>183</v>
       </c>
       <c r="E13" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F13" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B14">
         <v>30</v>
@@ -2709,15 +2712,15 @@
         <v>157</v>
       </c>
       <c r="E14" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="F14" t="s">
-        <v>190</v>
+        <v>402</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B15">
         <v>6</v>
@@ -2732,12 +2735,12 @@
         <v>158</v>
       </c>
       <c r="F15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B16">
         <v>3</v>
@@ -2752,12 +2755,12 @@
         <v>159</v>
       </c>
       <c r="F16" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2769,15 +2772,15 @@
         <v>51</v>
       </c>
       <c r="E17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F17" t="s">
-        <v>191</v>
+        <v>403</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B18">
         <v>-20</v>
@@ -2789,15 +2792,15 @@
         <v>183</v>
       </c>
       <c r="E18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F18" t="s">
-        <v>191</v>
+        <v>403</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B19">
         <v>20</v>
@@ -2809,15 +2812,15 @@
         <v>183</v>
       </c>
       <c r="E19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F19" t="s">
-        <v>191</v>
+        <v>403</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B20">
         <v>30</v>
@@ -2829,15 +2832,15 @@
         <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F20" t="s">
-        <v>191</v>
+        <v>403</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B21">
         <v>130</v>
@@ -2849,15 +2852,15 @@
         <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F21" t="s">
-        <v>191</v>
+        <v>403</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -2869,15 +2872,15 @@
         <v>51</v>
       </c>
       <c r="E22" t="s">
+        <v>206</v>
+      </c>
+      <c r="F22" t="s">
         <v>208</v>
-      </c>
-      <c r="F22" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B23">
         <v>3</v>
@@ -2889,10 +2892,10 @@
         <v>51</v>
       </c>
       <c r="E23" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F23" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2917,13 +2920,13 @@
   <sheetData>
     <row r="2" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="J2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="X2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.2">
@@ -2934,12 +2937,12 @@
         <v>9</v>
       </c>
       <c r="X3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -2960,7 +2963,7 @@
         <v>100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
@@ -2999,7 +3002,7 @@
         <v>250</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y4" s="1">
         <v>0</v>
@@ -3019,7 +3022,7 @@
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C5" s="1">
         <v>42</v>
@@ -3040,7 +3043,7 @@
         <v>11</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="K5" s="1">
         <v>360</v>
@@ -3079,7 +3082,7 @@
         <v>60</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="Y5" s="17">
         <v>50</v>
@@ -3099,7 +3102,7 @@
     </row>
     <row r="6" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
@@ -3120,7 +3123,7 @@
         <v>80</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -3159,7 +3162,7 @@
         <v>80</v>
       </c>
       <c r="X6" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y6" s="14">
         <v>0</v>
@@ -3179,7 +3182,7 @@
     </row>
     <row r="7" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C7" s="1">
         <v>12</v>
@@ -3200,7 +3203,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="K7" s="1">
         <v>220</v>
@@ -3239,7 +3242,7 @@
         <v>55</v>
       </c>
       <c r="X7" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="Y7" s="18">
         <v>60</v>
@@ -3259,7 +3262,7 @@
     </row>
     <row r="8" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C8" s="14">
         <v>5</v>
@@ -3280,7 +3283,7 @@
         <v>80</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K8" s="14">
         <v>5</v>
@@ -3326,7 +3329,7 @@
     </row>
     <row r="9" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C9" s="14">
         <v>40</v>
@@ -3347,7 +3350,7 @@
         <v>18</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="K9" s="14">
         <v>430</v>
@@ -3409,7 +3412,7 @@
     </row>
     <row r="13" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="Y13" s="16"/>
       <c r="Z13" s="16"/>
@@ -3430,7 +3433,7 @@
     </row>
     <row r="15" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C15" s="1">
         <v>5</v>
@@ -3451,7 +3454,7 @@
         <v>100</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K15" s="1">
         <v>5</v>
@@ -3478,7 +3481,7 @@
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="X15" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y15" s="1">
         <v>0</v>
@@ -3498,7 +3501,7 @@
     </row>
     <row r="16" spans="2:29" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C16" s="1">
         <v>4</v>
@@ -3519,7 +3522,7 @@
         <v>4</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="K16" s="1">
         <v>100</v>
@@ -3546,7 +3549,7 @@
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
       <c r="X16" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="Y16" s="1">
         <v>20</v>
@@ -3566,7 +3569,7 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C17" s="1">
         <v>5</v>
@@ -3587,7 +3590,7 @@
         <v>80</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="K17" s="14">
         <v>0</v>
@@ -3626,7 +3629,7 @@
         <v>80</v>
       </c>
       <c r="X17" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y17" s="14">
         <v>0</v>
@@ -3646,7 +3649,7 @@
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C18" s="1">
         <v>1.7</v>
@@ -3667,7 +3670,7 @@
         <v>5.2</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="K18" s="14">
         <v>580</v>
@@ -3706,7 +3709,7 @@
         <v>240</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="Y18" s="14">
         <v>55</v>
@@ -3726,7 +3729,7 @@
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B19" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C19" s="14">
         <v>5</v>
@@ -3749,7 +3752,7 @@
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B20" s="14" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C20" s="14">
         <v>2.8</v>
@@ -3772,12 +3775,12 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X24" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X25" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y25" s="1">
         <v>0</v>
@@ -3803,7 +3806,7 @@
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.2">
       <c r="X26" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="Y26" s="17">
         <v>2</v>
@@ -3898,7 +3901,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>22</v>
@@ -3936,7 +3939,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>22</v>
@@ -3974,7 +3977,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>22</v>
@@ -4469,7 +4472,7 @@
         <v>177</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>179</v>
@@ -4490,7 +4493,7 @@
         <v>7</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>14</v>
@@ -4507,10 +4510,10 @@
         <v>177</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
@@ -4519,7 +4522,7 @@
         <v>80</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="G18" s="1" t="b">
         <v>1</v>
@@ -4528,7 +4531,7 @@
         <v>7</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>14</v>
@@ -4545,10 +4548,10 @@
         <v>177</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D19" s="2">
         <v>-6</v>
@@ -4566,7 +4569,7 @@
         <v>7</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>14</v>
@@ -4583,10 +4586,10 @@
         <v>177</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>224</v>
       </c>
       <c r="D20" s="2">
         <v>0</v>
@@ -4595,7 +4598,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="G20" s="1" t="b">
         <v>1</v>
@@ -4604,7 +4607,7 @@
         <v>7</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>14</v>
@@ -4621,10 +4624,10 @@
         <v>91</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D21" s="2">
         <v>0</v>
@@ -4642,7 +4645,7 @@
         <v>7</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>14</v>
@@ -4656,13 +4659,13 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D22" s="2">
         <v>-10</v>
@@ -4680,7 +4683,7 @@
         <v>7</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>14</v>
@@ -4694,13 +4697,13 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>249</v>
       </c>
       <c r="D23" s="2">
         <v>-10</v>
@@ -4718,7 +4721,7 @@
         <v>7</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>14</v>
@@ -4732,13 +4735,13 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D24" s="2">
         <v>-10</v>
@@ -4756,7 +4759,7 @@
         <v>7</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>14</v>
@@ -4770,13 +4773,13 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D25" s="2">
         <v>-10</v>
@@ -4794,7 +4797,7 @@
         <v>7</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="J25" s="1" t="s">
         <v>14</v>
@@ -5504,7 +5507,7 @@
         <v>177</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D38" s="11" t="s">
         <v>70</v>
@@ -5513,7 +5516,7 @@
         <v>51</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
@@ -5521,7 +5524,7 @@
         <v>177</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>70</v>
@@ -5530,7 +5533,7 @@
         <v>51</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.2">
@@ -5538,7 +5541,7 @@
         <v>177</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>70</v>
@@ -5558,7 +5561,7 @@
         <v>177</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>70</v>
@@ -5578,14 +5581,14 @@
         <v>177</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>157</v>
       </c>
       <c r="E42" s="11"/>
       <c r="G42" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="43" spans="2:7" ht="96" x14ac:dyDescent="0.2">
@@ -5593,7 +5596,7 @@
         <v>177</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D43" s="11" t="s">
         <v>70</v>
@@ -5602,10 +5605,10 @@
         <v>51</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.2">
@@ -5613,7 +5616,7 @@
         <v>91</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>70</v>
@@ -5622,15 +5625,15 @@
         <v>51</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>70</v>
@@ -5639,15 +5642,15 @@
         <v>90</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="C46" s="12" t="s">
         <v>247</v>
-      </c>
-      <c r="C46" s="12" t="s">
-        <v>249</v>
       </c>
       <c r="D46" s="12" t="s">
         <v>70</v>
@@ -5656,15 +5659,15 @@
         <v>90</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D47" s="12" t="s">
         <v>70</v>
@@ -5673,15 +5676,15 @@
         <v>90</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" s="12" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>70</v>
@@ -5690,7 +5693,7 @@
         <v>90</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -5735,7 +5738,7 @@
         <v>188</v>
       </c>
       <c r="E2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -5743,7 +5746,7 @@
         <v>186</v>
       </c>
       <c r="B3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C3" t="s">
         <v>188</v>
@@ -5754,7 +5757,7 @@
         <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C4" t="s">
         <v>70</v>
@@ -5763,7 +5766,7 @@
         <v>77</v>
       </c>
       <c r="E4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -5771,7 +5774,7 @@
         <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C5" t="s">
         <v>70</v>
@@ -5785,7 +5788,7 @@
         <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C6" t="s">
         <v>70</v>
@@ -5799,7 +5802,7 @@
         <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C7" t="s">
         <v>70</v>
@@ -5813,7 +5816,7 @@
         <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C8" t="s">
         <v>70</v>
@@ -5827,7 +5830,7 @@
         <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C9" t="s">
         <v>70</v>
@@ -5841,7 +5844,7 @@
         <v>91</v>
       </c>
       <c r="B10" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C10" t="s">
         <v>70</v>
@@ -5855,7 +5858,7 @@
         <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C11" t="s">
         <v>70</v>
@@ -5869,7 +5872,7 @@
         <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C12" t="s">
         <v>70</v>
@@ -5883,7 +5886,7 @@
         <v>177</v>
       </c>
       <c r="B13" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -5892,7 +5895,7 @@
         <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>268</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -5900,7 +5903,7 @@
         <v>177</v>
       </c>
       <c r="B14" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C14" t="s">
         <v>70</v>
@@ -5914,7 +5917,7 @@
         <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" t="s">
         <v>70</v>
@@ -5928,7 +5931,7 @@
         <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C16" t="s">
         <v>70</v>
@@ -5942,7 +5945,7 @@
         <v>177</v>
       </c>
       <c r="B17" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C17" t="s">
         <v>70</v>
@@ -5956,7 +5959,7 @@
         <v>177</v>
       </c>
       <c r="B18" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C18" t="s">
         <v>70</v>
@@ -5970,7 +5973,7 @@
         <v>177</v>
       </c>
       <c r="B19" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C19" t="s">
         <v>70</v>
@@ -5984,7 +5987,7 @@
         <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" t="s">
         <v>70</v>
@@ -5998,7 +6001,7 @@
         <v>177</v>
       </c>
       <c r="B21" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C21" t="s">
         <v>70</v>

</xml_diff>

<commit_message>
add post-fix FromNdas to signals from DIStatus
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8C32DF-EC28-A647-856B-5C2CB3E99585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F7D606-5FB9-344D-9D02-3B05E72AC53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37360" yWindow="2220" windowWidth="31940" windowHeight="19140" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="10" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="cycleKPI" sheetId="8" r:id="rId6"/>
     <sheet name="markerShapes" sheetId="5" r:id="rId7"/>
     <sheet name="lineColors" sheetId="4" r:id="rId8"/>
+    <sheet name="GT" sheetId="12" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="419">
   <si>
     <t>Reference</t>
   </si>
@@ -1125,57 +1126,30 @@
     <t>active_safety_status/settings/AEB/actuation_precondition_blocked</t>
   </si>
   <si>
-    <t>aebPrecondBlk</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/AEB/abort_any_active_events</t>
   </si>
   <si>
-    <t>aebAbort</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/FCW/warning_precondition_blocked</t>
   </si>
   <si>
-    <t>fcwPrecondBlk</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/FCW/abort_any_active_events</t>
   </si>
   <si>
-    <t>fcwAbort</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/DBS/actuation_precondition_blocked</t>
   </si>
   <si>
-    <t>ebaPrecondBlk</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/DBS/abort_any_active_events</t>
   </si>
   <si>
-    <t>ebaAbort</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/CPM/actuation_precondition_blocked</t>
   </si>
   <si>
-    <t>cpmActPrecondBlk</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/CPM/warning_precondition_blocked</t>
   </si>
   <si>
-    <t>cpmWrnPrecondBlk</t>
-  </si>
-  <si>
     <t>active_safety_status/settings/CPM/abort_any_active_events</t>
   </si>
   <si>
-    <t>cpmAbort</t>
-  </si>
-  <si>
     <t>gpsFrame</t>
   </si>
   <si>
@@ -1261,6 +1235,75 @@
   </si>
   <si>
     <t>fcw availability</t>
+  </si>
+  <si>
+    <t>gtFlag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longitudinal gap between ego and target </t>
+  </si>
+  <si>
+    <t>lateral gap between ego and target</t>
+  </si>
+  <si>
+    <t>time to collision</t>
+  </si>
+  <si>
+    <t>boolean signal that represent the FCW audio alert</t>
+  </si>
+  <si>
+    <t>longGapGT</t>
+  </si>
+  <si>
+    <t>latGapGT</t>
+  </si>
+  <si>
+    <t>ttcGT</t>
+  </si>
+  <si>
+    <t>audioGT</t>
+  </si>
+  <si>
+    <t>GTName</t>
+  </si>
+  <si>
+    <t>Processing method</t>
+  </si>
+  <si>
+    <t>req-5256401-00201489</t>
+  </si>
+  <si>
+    <t>aebSuspDur</t>
+  </si>
+  <si>
+    <t>when the system is overriden, the system shall suspend AEB from initiating another braking for 5s</t>
+  </si>
+  <si>
+    <t>aebAbortFromNdas</t>
+  </si>
+  <si>
+    <t>fcwAbortFromNdas</t>
+  </si>
+  <si>
+    <t>ebaAbortFromNdas</t>
+  </si>
+  <si>
+    <t>cpmActPrecondBlkFromNdas</t>
+  </si>
+  <si>
+    <t>cpmWrnPrecondBlkFromNdas</t>
+  </si>
+  <si>
+    <t>cpmAbortFromNdas</t>
+  </si>
+  <si>
+    <t>aebPrecondBlkFromNdas</t>
+  </si>
+  <si>
+    <t>fcwPrecondBlkFromNdas</t>
+  </si>
+  <si>
+    <t>ebaPrecondBlkFromNdas</t>
   </si>
 </sst>
 </file>
@@ -1703,17 +1746,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4532B10-0F66-F744-8436-DE50D0D74792}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="53.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.5" customWidth="1"/>
     <col min="4" max="4" width="5.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>288</v>
       </c>
@@ -1729,8 +1772,11 @@
       <c r="E1" s="5" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" s="5" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>291</v>
       </c>
@@ -1744,7 +1790,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>291</v>
       </c>
@@ -1758,7 +1804,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>296</v>
       </c>
@@ -1775,7 +1821,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>300</v>
       </c>
@@ -1792,7 +1838,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>300</v>
       </c>
@@ -1806,7 +1852,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>306</v>
       </c>
@@ -1820,7 +1866,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>309</v>
       </c>
@@ -1834,7 +1880,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>300</v>
       </c>
@@ -1851,7 +1897,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>309</v>
       </c>
@@ -1868,7 +1914,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>291</v>
       </c>
@@ -1885,7 +1931,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>320</v>
       </c>
@@ -1898,8 +1944,11 @@
       <c r="D12" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>320</v>
       </c>
@@ -1913,7 +1962,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>320</v>
       </c>
@@ -1927,7 +1976,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>320</v>
       </c>
@@ -1940,8 +1989,11 @@
       <c r="D15" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>320</v>
       </c>
@@ -1955,7 +2007,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>320</v>
       </c>
@@ -1969,7 +2021,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>320</v>
       </c>
@@ -1983,7 +2035,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>300</v>
       </c>
@@ -1997,7 +2049,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>338</v>
       </c>
@@ -2011,7 +2063,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>338</v>
       </c>
@@ -2025,7 +2077,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>338</v>
       </c>
@@ -2039,7 +2091,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>344</v>
       </c>
@@ -2053,7 +2105,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>344</v>
       </c>
@@ -2067,7 +2119,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>320</v>
       </c>
@@ -2080,8 +2132,11 @@
       <c r="D25" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>344</v>
       </c>
@@ -2095,7 +2150,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>353</v>
       </c>
@@ -2108,8 +2163,11 @@
       <c r="D27" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>353</v>
       </c>
@@ -2122,8 +2180,11 @@
       <c r="D28" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>344</v>
       </c>
@@ -2131,49 +2192,49 @@
         <v>358</v>
       </c>
       <c r="C29" t="s">
-        <v>359</v>
+        <v>416</v>
       </c>
       <c r="D29" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>344</v>
       </c>
       <c r="B30" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C30" t="s">
-        <v>361</v>
+        <v>410</v>
       </c>
       <c r="D30" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>344</v>
       </c>
       <c r="B31" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C31" t="s">
-        <v>363</v>
+        <v>417</v>
       </c>
       <c r="D31" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>344</v>
       </c>
       <c r="B32" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C32" t="s">
-        <v>365</v>
+        <v>411</v>
       </c>
       <c r="D32" t="s">
         <v>157</v>
@@ -2184,10 +2245,10 @@
         <v>344</v>
       </c>
       <c r="B33" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="C33" t="s">
-        <v>367</v>
+        <v>418</v>
       </c>
       <c r="D33" t="s">
         <v>157</v>
@@ -2198,10 +2259,10 @@
         <v>344</v>
       </c>
       <c r="B34" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C34" t="s">
-        <v>369</v>
+        <v>412</v>
       </c>
       <c r="D34" t="s">
         <v>157</v>
@@ -2212,10 +2273,10 @@
         <v>344</v>
       </c>
       <c r="B35" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="C35" t="s">
-        <v>371</v>
+        <v>413</v>
       </c>
       <c r="D35" t="s">
         <v>157</v>
@@ -2226,10 +2287,10 @@
         <v>344</v>
       </c>
       <c r="B36" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="C36" t="s">
-        <v>373</v>
+        <v>414</v>
       </c>
       <c r="D36" t="s">
         <v>157</v>
@@ -2240,10 +2301,10 @@
         <v>344</v>
       </c>
       <c r="B37" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="C37" t="s">
-        <v>375</v>
+        <v>415</v>
       </c>
       <c r="D37" t="s">
         <v>157</v>
@@ -2251,13 +2312,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="B38" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="C38" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="D38" t="s">
         <v>147</v>
@@ -2265,13 +2326,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="B39" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="C39" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="D39" t="s">
         <v>147</v>
@@ -2282,10 +2343,10 @@
         <v>320</v>
       </c>
       <c r="B40" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="C40" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="D40" t="s">
         <v>157</v>
@@ -2296,10 +2357,10 @@
         <v>320</v>
       </c>
       <c r="B41" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="C41" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="D41" t="s">
         <v>157</v>
@@ -2310,10 +2371,10 @@
         <v>344</v>
       </c>
       <c r="B42" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="C42" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="D42" t="s">
         <v>331</v>
@@ -2324,10 +2385,10 @@
         <v>344</v>
       </c>
       <c r="B43" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="C43" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="D43" t="s">
         <v>331</v>
@@ -2338,10 +2399,10 @@
         <v>344</v>
       </c>
       <c r="B44" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="C44" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="D44" t="s">
         <v>331</v>
@@ -2352,10 +2413,10 @@
         <v>344</v>
       </c>
       <c r="B45" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="C45" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="D45" t="s">
         <v>331</v>
@@ -2363,13 +2424,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="B46" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="C46" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="D46" t="s">
         <v>147</v>
@@ -2377,13 +2438,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="B47" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="C47" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="D47" t="s">
         <v>147</v>
@@ -2391,13 +2452,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="B48" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="C48" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="D48" t="s">
         <v>147</v>
@@ -2408,10 +2469,10 @@
         <v>320</v>
       </c>
       <c r="B49" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="C49" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="D49" t="s">
         <v>157</v>
@@ -2422,10 +2483,10 @@
         <v>320</v>
       </c>
       <c r="B50" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="C50" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
       <c r="D50" t="s">
         <v>331</v>
@@ -2529,7 +2590,7 @@
         <v>210</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
         <v>147</v>
@@ -2558,7 +2619,7 @@
         <v>237</v>
       </c>
       <c r="F6" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -2578,7 +2639,7 @@
         <v>153</v>
       </c>
       <c r="F7" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -2598,7 +2659,7 @@
         <v>154</v>
       </c>
       <c r="F8" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -2618,7 +2679,7 @@
         <v>239</v>
       </c>
       <c r="F9" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2638,7 +2699,7 @@
         <v>155</v>
       </c>
       <c r="F10" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -2658,7 +2719,7 @@
         <v>156</v>
       </c>
       <c r="F11" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -2678,7 +2739,7 @@
         <v>231</v>
       </c>
       <c r="F12" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -2698,7 +2759,7 @@
         <v>243</v>
       </c>
       <c r="F13" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -2715,7 +2776,7 @@
         <v>235</v>
       </c>
       <c r="F14" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -2775,7 +2836,7 @@
         <v>191</v>
       </c>
       <c r="F17" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -2795,7 +2856,7 @@
         <v>232</v>
       </c>
       <c r="F18" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -2815,7 +2876,7 @@
         <v>233</v>
       </c>
       <c r="F19" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -2835,7 +2896,7 @@
         <v>202</v>
       </c>
       <c r="F20" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -2855,7 +2916,7 @@
         <v>203</v>
       </c>
       <c r="F21" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -4830,7 +4891,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE39B99-0AFB-8547-83BF-D855CC6E3BB3}">
-  <dimension ref="B1:G48"/>
+  <dimension ref="B1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="12" customWidth="1"/>
@@ -5694,6 +5755,26 @@
       </c>
       <c r="G48" s="12" t="s">
         <v>253</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B49" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="G49" s="12" t="s">
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -5895,7 +5976,7 @@
         <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -6218,4 +6299,63 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB8588E0-9289-B54C-B4B4-9C13CBC4F7E8}">
+  <dimension ref="B1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>402</v>
+      </c>
+      <c r="C3" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>403</v>
+      </c>
+      <c r="C4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" t="s">
+        <v>400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
KPI: aeb override suspension duration added
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F7D606-5FB9-344D-9D02-3B05E72AC53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C306696-E431-BA43-A6CD-3FEC4D20D3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="10" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="421">
   <si>
     <t>Reference</t>
   </si>
@@ -1304,6 +1304,12 @@
   </si>
   <si>
     <t>ebaPrecondBlkFromNdas</t>
+  </si>
+  <si>
+    <t>AEB Suspension Duration</t>
+  </si>
+  <si>
+    <t>AEB OverrideSuspDuration</t>
   </si>
 </sst>
 </file>
@@ -4871,18 +4877,42 @@
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
+      <c r="A26" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1">
+        <v>10</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G26" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" s="1" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add obj velocity to the signal list and calculate the relative impact speed
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C306696-E431-BA43-A6CD-3FEC4D20D3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E170C28C-A2A3-504F-A5DA-DC1DEE751989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="10" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="426">
   <si>
     <t>Reference</t>
   </si>
@@ -1310,6 +1310,23 @@
   </si>
   <si>
     <t>AEB OverrideSuspDuration</t>
+  </si>
+  <si>
+    <t>req-5256401-00191355
+req-5256401-00191360
+req-5256401-00191361</t>
+  </si>
+  <si>
+    <t>relative speed between ego and target the moment a collision happens</t>
+  </si>
+  <si>
+    <t>ImpactRelSpdKph</t>
+  </si>
+  <si>
+    <t>obstacle/velocity_mps/x</t>
+  </si>
+  <si>
+    <t>objSpeed</t>
   </si>
 </sst>
 </file>
@@ -1752,7 +1769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4532B10-0F66-F744-8436-DE50D0D74792}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
@@ -2470,7 +2487,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>320</v>
       </c>
@@ -2484,7 +2501,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>320</v>
       </c>
@@ -2496,6 +2513,23 @@
       </c>
       <c r="D50" t="s">
         <v>331</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>382</v>
+      </c>
+      <c r="B51" t="s">
+        <v>424</v>
+      </c>
+      <c r="C51" t="s">
+        <v>425</v>
+      </c>
+      <c r="D51" t="s">
+        <v>147</v>
+      </c>
+      <c r="E51" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -4921,7 +4955,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE39B99-0AFB-8547-83BF-D855CC6E3BB3}">
-  <dimension ref="B1:G49"/>
+  <dimension ref="B1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="12" customWidth="1"/>
@@ -5805,6 +5839,26 @@
       </c>
       <c r="G49" s="12" t="s">
         <v>409</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" ht="48" x14ac:dyDescent="0.2">
+      <c r="B50" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>423</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>421</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
aeb degradation check implemented
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E170C28C-A2A3-504F-A5DA-DC1DEE751989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35013CF-CC88-B449-8C8A-1C7A05F19529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="430">
   <si>
     <t>Reference</t>
   </si>
@@ -1327,6 +1327,18 @@
   </si>
   <si>
     <t>objSpeed</t>
+  </si>
+  <si>
+    <t>NoDegradation</t>
+  </si>
+  <si>
+    <t>mileage ratio of no degradation</t>
+  </si>
+  <si>
+    <t>fcw_state_info/degradation</t>
+  </si>
+  <si>
+    <t>fcwDegradation</t>
   </si>
 </sst>
 </file>
@@ -1769,7 +1781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4532B10-0F66-F744-8436-DE50D0D74792}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
@@ -2530,6 +2542,20 @@
       </c>
       <c r="E51" t="s">
         <v>303</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>320</v>
+      </c>
+      <c r="B52" t="s">
+        <v>428</v>
+      </c>
+      <c r="C52" t="s">
+        <v>429</v>
+      </c>
+      <c r="D52" t="s">
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -5868,7 +5894,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5705F2F5-A4FE-CE49-A935-9D51D28B5CFA}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -6048,10 +6074,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>264</v>
+        <v>426</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -6060,7 +6086,7 @@
         <v>77</v>
       </c>
       <c r="E13" t="s">
-        <v>395</v>
+        <v>427</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -6068,13 +6094,16 @@
         <v>177</v>
       </c>
       <c r="B14" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="C14" t="s">
         <v>70</v>
       </c>
       <c r="D14" t="s">
         <v>77</v>
+      </c>
+      <c r="E14" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -6082,7 +6111,7 @@
         <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C15" t="s">
         <v>70</v>
@@ -6096,7 +6125,7 @@
         <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C16" t="s">
         <v>70</v>
@@ -6110,7 +6139,7 @@
         <v>177</v>
       </c>
       <c r="B17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C17" t="s">
         <v>70</v>
@@ -6124,7 +6153,7 @@
         <v>177</v>
       </c>
       <c r="B18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C18" t="s">
         <v>70</v>
@@ -6138,7 +6167,7 @@
         <v>177</v>
       </c>
       <c r="B19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C19" t="s">
         <v>70</v>
@@ -6152,7 +6181,7 @@
         <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C20" t="s">
         <v>70</v>
@@ -6166,12 +6195,40 @@
         <v>177</v>
       </c>
       <c r="B21" t="s">
+        <v>286</v>
+      </c>
+      <c r="C21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>177</v>
+      </c>
+      <c r="B22" t="s">
         <v>287</v>
       </c>
-      <c r="C21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" t="s">
+        <v>426</v>
+      </c>
+      <c r="C23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fcw degradation check implemented
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35013CF-CC88-B449-8C8A-1C7A05F19529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91F5DB1-7AB1-2D42-A96E-9FD71DAE7A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="34200" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vbRcSignals" sheetId="10" r:id="rId1"/>

</xml_diff>

<commit_message>
Plot LSAEB average acceleration magnitude
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -3291,7 +3291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12.5" customWidth="1" min="1" max="1"/>
@@ -4673,106 +4673,158 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LSAEB</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>LSAEB Average Acceleration Magnitude</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>abs(lsaebAverageAccel)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Acceleration Magnitude (m/s2)</t>
+        </is>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LSAEB Average Acceleration Magnitude</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>scatter</t>
+        </is>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>AEB</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>AEB Suspension Duration</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>aebSuspDur</t>
         </is>
       </c>
-      <c r="D27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="1" t="n">
+      <c r="D28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>Time (sec)</t>
         </is>
       </c>
-      <c r="G27" s="1" t="b">
+      <c r="G28" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="H27" s="1" t="inlineStr">
+      <c r="H28" s="1" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="I27" s="1" t="inlineStr">
+      <c r="I28" s="1" t="inlineStr">
         <is>
           <t>AEB OverrideSuspDuration</t>
         </is>
       </c>
-      <c r="J27" s="1" t="inlineStr">
+      <c r="J28" s="1" t="inlineStr">
         <is>
           <t>scatter</t>
         </is>
       </c>
-      <c r="K27" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="L27" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="K28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>AEB</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>AEB Stop Distance</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>brakeDistAeb</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>4000</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Distance (cm)</t>
         </is>
       </c>
-      <c r="G28" t="b">
+      <c r="G29" t="b">
         <v>1</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>AEB Stop Distance</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>scatter</t>
         </is>
       </c>
-      <c r="K28" t="b">
-        <v>0</v>
-      </c>
-      <c r="L28" t="b">
+      <c r="K29" t="b">
+        <v>0</v>
+      </c>
+      <c r="L29" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Start average accel at actual decel onset
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -4839,7 +4839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="2.83203125" customWidth="1" style="12" min="1" max="1"/>
@@ -6254,6 +6254,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
@@ -6277,7 +6278,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Average longActAccel from the first autonomous braking edge to egoSpeedKph &lt; 0.05 for AEB events (&gt;10 kph start speed)</t>
+          <t>Average longActAccel from actual deceleration onset to egoSpeedKph &lt; 0.05 for AEB events (&gt;10 kph start speed)</t>
         </is>
       </c>
     </row>
@@ -6331,7 +6332,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Average longActAccel from the first autonomous braking edge to egoSpeedKph &lt; 0.05 for LSAEB events ((2,10] kph start speed)</t>
+          <t>Average longActAccel from actual deceleration onset to egoSpeedKph &lt; 0.05 for LSAEB events ((2,10] kph start speed)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust average acceleration plot ranges
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -3291,7 +3291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12.5" customWidth="1" min="1" max="1"/>
@@ -4692,7 +4692,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4825,6 +4825,58 @@
         <v>0</v>
       </c>
       <c r="L29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AEB</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AEB Average Acceleration Magnitude</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>abs(aebAverageAccel)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>15</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Acceleration Magnitude (m/s2)</t>
+        </is>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>AEB Average Acceleration Magnitude</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>scatter</t>
+        </is>
+      </c>
+      <c r="K30" t="b">
+        <v>0</v>
+      </c>
+      <c r="L30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4839,7 +4891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="B1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="2.83203125" customWidth="1" style="12" min="1" max="1"/>
@@ -6254,7 +6306,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Start brake distance at actual decel onset
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -4891,7 +4891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="2.83203125" customWidth="1" style="12" min="1" max="1"/>
@@ -6306,6 +6306,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
@@ -6356,7 +6357,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Integrated egoSpeed from the first aebTargetDecel falling edge to egoSpeed == 0 for AEB events</t>
+          <t>Integrated egoSpeed from actual deceleration onset to egoSpeed == 0 for AEB events</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6411,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Integrated egoSpeed from the first aebTargetDecel falling edge to egoSpeed == 0 for LSAEB events</t>
+          <t>Integrated egoSpeed from actual deceleration onset to egoSpeed == 0 for LSAEB events</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add MOTION_1 MF4 processing
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -366,22 +366,27 @@
           <t>synonym</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MOTION_1</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>genericName</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>gtFlag</t>
         </is>
@@ -398,12 +403,12 @@
           <t>acceleration[1]</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>latActAccel</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -422,10 +427,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>longActAccel</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -444,15 +454,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>DADCAxLmtIT4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>aebTargetDecel</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>m/s2</t>
         </is>
@@ -471,15 +486,20 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>VehicleSpeed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>egoSpeed</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -498,10 +518,15 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>PedalPosPro</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>throttleValue</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -518,12 +543,12 @@
           <t>active_safety_settings/AEB/abort_any_active_events</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>aebAbortFromVcs</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -542,10 +567,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>BrakeSwitchStatus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>brakePedalPressed</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -564,15 +594,20 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>SteeringWheelAngle</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>steerWheelAngle</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>rad</t>
         </is>
@@ -591,15 +626,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>SteeringWheelAngleSpeed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>steerWheelAngleSpeed</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>rad/s</t>
         </is>
@@ -618,15 +658,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>YawRate</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>yawRate</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>rad/s</t>
         </is>
@@ -643,17 +688,17 @@
           <t>aeb_state_info/aeb_full_state_info/longitudinal_clearance</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>longGap</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F12" t="b">
+      <c r="G12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -668,12 +713,12 @@
           <t>aeb_state_info/most_relevant_object_id</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>aebTargetId</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -690,12 +735,12 @@
           <t>fcw_state_info/most_relevant_object_id</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>fcwTargetId</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -712,17 +757,17 @@
           <t>aeb_state_info/time_to_collision</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>aebTTC</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F15" t="b">
+      <c r="G15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -737,12 +782,12 @@
           <t>aeb_state_info/aeb_full_state_info/state</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>aebFullState</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -759,12 +804,12 @@
           <t>aeb_state_info/aeb_partial_state_info/state</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>aebPartialState</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -783,10 +828,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>FCWState</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>fcwState</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -803,12 +853,12 @@
           <t>vehicle_stopped</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>isVehStoppedNV</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -825,12 +875,12 @@
           <t>fcw_request</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>fcwRequest</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -847,12 +897,12 @@
           <t>aeb_request</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>aebRequest</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -869,12 +919,12 @@
           <t>dbs_request</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>dbsRequest</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -891,12 +941,12 @@
           <t>active_safety_status/settings/FCW/configuration_level</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>fcwSensitivity</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -913,12 +963,12 @@
           <t>active_safety_settings/AEB/configuration_level</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>aebConfigLvl</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -935,17 +985,17 @@
           <t>fcw_state_info/time_to_collision</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>fcwTTC</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F25" t="b">
+      <c r="G25" t="b">
         <v>1</v>
       </c>
     </row>
@@ -960,12 +1010,12 @@
           <t>active_safety_status/notices/CPM/braking_event_status</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>cpmEventType</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -982,17 +1032,17 @@
           <t>daa_state_info/obstruction_position/x</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>cpmLongDist</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F27" t="b">
+      <c r="G27" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1007,17 +1057,17 @@
           <t>daa_state_info/obstruction_position/y</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>cpmLatDist</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F28" t="b">
+      <c r="G28" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1032,12 +1082,12 @@
           <t>active_safety_status/settings/AEB/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>aebPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1054,12 +1104,12 @@
           <t>active_safety_status/settings/AEB/abort_any_active_events</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>aebAbortFromNdas</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1076,12 +1126,12 @@
           <t>active_safety_status/settings/FCW/warning_precondition_blocked</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>fcwPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1098,12 +1148,12 @@
           <t>active_safety_status/settings/FCW/abort_any_active_events</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>fcwAbortFromNdas</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1120,12 +1170,12 @@
           <t>active_safety_status/settings/DBS/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>ebaPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1142,12 +1192,12 @@
           <t>active_safety_status/settings/DBS/abort_any_active_events</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>ebaAbortFromNdas</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1164,12 +1214,12 @@
           <t>active_safety_status/settings/CPM/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>cpmActPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1186,12 +1236,12 @@
           <t>active_safety_status/settings/CPM/warning_precondition_blocked</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>cpmWrnPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1208,12 +1258,12 @@
           <t>active_safety_status/settings/CPM/abort_any_active_events</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>cpmAbortFromNdas</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1230,12 +1280,12 @@
           <t>latitude</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1252,12 +1302,12 @@
           <t>longitude</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1274,12 +1324,12 @@
           <t>is_input_healthy</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>aebInputHealthy</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1296,12 +1346,12 @@
           <t>cpm_state_info/is_input_healthy</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>cpmInputHealthy</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1318,12 +1368,12 @@
           <t>active_safety_status/settings/CPM/run_setting</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>cpmRunSetting</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1340,12 +1390,12 @@
           <t>active_safety_status/settings/FCW/run_setting</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>fcwRunSetting</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1362,12 +1412,12 @@
           <t>active_safety_status/settings/AEB/run_setting</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>aebRunSetting</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1384,12 +1434,12 @@
           <t>active_safety_status/settings/DBS/run_setting</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>dbsRunSetting</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1406,12 +1456,12 @@
           <t>obstacle/confidence</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>obstConf</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1428,12 +1478,12 @@
           <t>obstacle/position_confidence/confidence</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>posConf</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1450,12 +1500,12 @@
           <t>obstacle/velocity_confidence/confidence</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>velConf</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1472,12 +1522,12 @@
           <t>target_obstacle_class</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>aebTargetType</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1494,12 +1544,12 @@
           <t>aeb_state_info/degradation</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>aebDegradation</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1516,17 +1566,17 @@
           <t>obstacle/velocity_mps/x</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>objSpeed</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -1543,12 +1593,12 @@
           <t>fcw_state_info/degradation</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>fcwDegradation</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -4891,7 +4941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="B1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="2.83203125" customWidth="1" style="12" min="1" max="1"/>
@@ -6306,7 +6356,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Clarify MOTION_1 source signal units
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -345,7 +345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -371,22 +371,27 @@
           <t>MOTION_1</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>MOTION_1_Unit</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>genericName</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>gtFlag</t>
         </is>
@@ -403,12 +408,12 @@
           <t>acceleration[1]</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>latActAccel</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -432,10 +437,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>m/s2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>longActAccel</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -459,15 +469,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>m/s2 command</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>aebTargetDecel</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>m/s2</t>
         </is>
@@ -491,15 +506,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>km/h</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>egoSpeed</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -523,10 +543,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>throttleValue</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -543,12 +568,12 @@
           <t>active_safety_settings/AEB/abort_any_active_events</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>aebAbortFromVcs</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -572,10 +597,15 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>brakePedalPressed</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -599,15 +629,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>deg</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>steerWheelAngle</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>rad</t>
         </is>
@@ -631,15 +666,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>deg/s</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>steerWheelAngleSpeed</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>rad/s</t>
         </is>
@@ -663,15 +703,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>deg/s</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>yawRate</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>rad/s</t>
         </is>
@@ -688,17 +733,17 @@
           <t>aeb_state_info/aeb_full_state_info/longitudinal_clearance</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>longGap</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="G12" t="b">
+      <c r="H12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -713,12 +758,12 @@
           <t>aeb_state_info/most_relevant_object_id</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>aebTargetId</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -735,12 +780,12 @@
           <t>fcw_state_info/most_relevant_object_id</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>fcwTargetId</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -757,17 +802,17 @@
           <t>aeb_state_info/time_to_collision</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>aebTTC</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="G15" t="b">
+      <c r="H15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -782,12 +827,12 @@
           <t>aeb_state_info/aeb_full_state_info/state</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>aebFullState</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -804,12 +849,12 @@
           <t>aeb_state_info/aeb_partial_state_info/state</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>aebPartialState</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -833,10 +878,15 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>fcwState</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -853,12 +903,12 @@
           <t>vehicle_stopped</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>isVehStoppedNV</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -875,12 +925,12 @@
           <t>fcw_request</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>fcwRequest</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -897,12 +947,12 @@
           <t>aeb_request</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>aebRequest</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -919,12 +969,12 @@
           <t>dbs_request</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>dbsRequest</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -941,12 +991,12 @@
           <t>active_safety_status/settings/FCW/configuration_level</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>fcwSensitivity</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -963,12 +1013,12 @@
           <t>active_safety_settings/AEB/configuration_level</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>aebConfigLvl</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -985,17 +1035,17 @@
           <t>fcw_state_info/time_to_collision</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>fcwTTC</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="G25" t="b">
+      <c r="H25" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1010,12 +1060,12 @@
           <t>active_safety_status/notices/CPM/braking_event_status</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>cpmEventType</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1032,17 +1082,17 @@
           <t>daa_state_info/obstruction_position/x</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>cpmLongDist</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="G27" t="b">
+      <c r="H27" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1057,17 +1107,17 @@
           <t>daa_state_info/obstruction_position/y</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>cpmLatDist</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="G28" t="b">
+      <c r="H28" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1082,12 +1132,12 @@
           <t>active_safety_status/settings/AEB/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>aebPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1104,12 +1154,12 @@
           <t>active_safety_status/settings/AEB/abort_any_active_events</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>aebAbortFromNdas</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1126,12 +1176,12 @@
           <t>active_safety_status/settings/FCW/warning_precondition_blocked</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>fcwPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1148,12 +1198,12 @@
           <t>active_safety_status/settings/FCW/abort_any_active_events</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>fcwAbortFromNdas</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1170,12 +1220,12 @@
           <t>active_safety_status/settings/DBS/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>ebaPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1192,12 +1242,12 @@
           <t>active_safety_status/settings/DBS/abort_any_active_events</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>ebaAbortFromNdas</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1214,12 +1264,12 @@
           <t>active_safety_status/settings/CPM/actuation_precondition_blocked</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>cpmActPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1236,12 +1286,12 @@
           <t>active_safety_status/settings/CPM/warning_precondition_blocked</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>cpmWrnPrecondBlkFromNdas</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1258,12 +1308,12 @@
           <t>active_safety_status/settings/CPM/abort_any_active_events</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>cpmAbortFromNdas</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1280,12 +1330,12 @@
           <t>latitude</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1302,12 +1352,12 @@
           <t>longitude</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1324,12 +1374,12 @@
           <t>is_input_healthy</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>aebInputHealthy</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1346,12 +1396,12 @@
           <t>cpm_state_info/is_input_healthy</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>cpmInputHealthy</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1368,12 +1418,12 @@
           <t>active_safety_status/settings/CPM/run_setting</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>cpmRunSetting</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1390,12 +1440,12 @@
           <t>active_safety_status/settings/FCW/run_setting</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>fcwRunSetting</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1412,12 +1462,12 @@
           <t>active_safety_status/settings/AEB/run_setting</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>aebRunSetting</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1434,12 +1484,12 @@
           <t>active_safety_status/settings/DBS/run_setting</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>dbsRunSetting</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1456,12 +1506,12 @@
           <t>obstacle/confidence</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>obstConf</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1478,12 +1528,12 @@
           <t>obstacle/position_confidence/confidence</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>posConf</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1500,12 +1550,12 @@
           <t>obstacle/velocity_confidence/confidence</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>velConf</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -1522,12 +1572,12 @@
           <t>target_obstacle_class</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>aebTargetType</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>int</t>
         </is>
@@ -1544,12 +1594,12 @@
           <t>aeb_state_info/degradation</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>aebDegradation</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
@@ -1566,17 +1616,17 @@
           <t>obstacle/velocity_mps/x</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>objSpeed</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -1593,12 +1643,12 @@
           <t>fcw_state_info/degradation</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>fcwDegradation</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>enum</t>
         </is>

</xml_diff>

<commit_message>
Add MOTION_1 lateral acceleration KPIs
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_long.xlsx
+++ b/src/config/kpi_as_long.xlsx
@@ -408,6 +408,16 @@
           <t>acceleration[1]</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>m/s2</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>latActAccel</t>

</xml_diff>